<commit_message>
se agrega la automatizacion de transacciones a terceros completa
</commit_message>
<xml_diff>
--- a/Banca en Linea modelo 2/Datos/Datos.xlsx
+++ b/Banca en Linea modelo 2/Datos/Datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bespinosa\Documents\Katalon\Demo Banca en Linea\Demo-Banca-en-Linea\Banca en Linea modelo 2\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9765C1FB-2404-4AD8-AB8B-6571D8CDB645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93769519-D9C4-454A-BE10-9EBF5FAAC7E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -393,7 +393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
@@ -450,54 +450,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>